<commit_message>
Add auto repair labour (трудозатраты) to supplier templates, as in the examples
Repair service cost is now computed like the source files: for each year, the
man-hours (нормо-час) of the components repaired that year x the service rate.
ТО service was already computed (ч·часы ТО x rate); repair service is carved out
of the capital-repair total so the annual ТОиР and annuities stay reconciled.
Example now shows non-zero labour in capital-repair years (e.g. PC2000-8 year 4:
ТО service 27.3 + repair service 12.5 = 39.8 тыс), total ТОиР unchanged (1430.6).

Validated: full workbook recalculates with zero errors; annuities unchanged
(PC2000-8 48.71 руб/м³).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WL5xBBk55GzPMRGQKQMRy3
</commit_message>
<xml_diff>
--- a/Модель_TCO_экскаваторов_аннуитет.xlsx
+++ b/Модель_TCO_экскаваторов_аннуитет.xlsx
@@ -3422,7 +3422,7 @@
     <row r="34">
       <c r="B34" s="37" t="inlineStr">
         <is>
-          <t>Капитальные ремонты (ППР) — из списка</t>
+          <t>Капитальные ремонты (запчасти) — авто</t>
         </is>
       </c>
       <c r="C34" s="24" t="inlineStr">
@@ -3431,50 +3431,50 @@
         </is>
       </c>
       <c r="E34" s="38">
-        <f>SUM(E69:E90)</f>
+        <f>SUM(E69:E90)-E35</f>
         <v/>
       </c>
       <c r="F34" s="38">
-        <f>SUM(F69:F90)</f>
+        <f>SUM(F69:F90)-F35</f>
         <v/>
       </c>
       <c r="G34" s="38">
-        <f>SUM(G69:G90)</f>
+        <f>SUM(G69:G90)-G35</f>
         <v/>
       </c>
       <c r="H34" s="38">
-        <f>SUM(H69:H90)</f>
+        <f>SUM(H69:H90)-H35</f>
         <v/>
       </c>
       <c r="I34" s="38">
-        <f>SUM(I69:I90)</f>
+        <f>SUM(I69:I90)-I35</f>
         <v/>
       </c>
       <c r="J34" s="38">
-        <f>SUM(J69:J90)</f>
+        <f>SUM(J69:J90)-J35</f>
         <v/>
       </c>
       <c r="K34" s="38">
-        <f>SUM(K69:K90)</f>
+        <f>SUM(K69:K90)-K35</f>
         <v/>
       </c>
       <c r="L34" s="38">
-        <f>SUM(L69:L90)</f>
+        <f>SUM(L69:L90)-L35</f>
         <v/>
       </c>
       <c r="M34" s="38">
-        <f>SUM(M69:M90)</f>
+        <f>SUM(M69:M90)-M35</f>
         <v/>
       </c>
       <c r="N34" s="38">
-        <f>SUM(N69:N90)</f>
+        <f>SUM(N69:N90)-N35</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="22" t="inlineStr">
-        <is>
-          <t>Сервис ремонтов (трудозатраты)</t>
+      <c r="B35" s="37" t="inlineStr">
+        <is>
+          <t>Сервис ремонтов (трудозатраты, авто)</t>
         </is>
       </c>
       <c r="C35" s="24" t="inlineStr">
@@ -3482,35 +3482,45 @@
           <t>тыс/год</t>
         </is>
       </c>
-      <c r="E35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" s="31" t="n">
-        <v>0</v>
+      <c r="E35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(E69:E90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="F35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(F69:F90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="G35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(G69:G90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="H35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(H69:H90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="I35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(I69:I90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="J35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(J69:J90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="K35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(K69:K90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="L35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(L69:L90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="M35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(M69:M90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="N35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(N69:N90&gt;0)*1)*$E$29/1000</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -4616,6 +4626,9 @@
           <t>Прочие/укрупнённо (капремонт)</t>
         </is>
       </c>
+      <c r="C90" s="47" t="n">
+        <v>250</v>
+      </c>
       <c r="E90" s="47" t="n">
         <v>0</v>
       </c>
@@ -4650,7 +4663,7 @@
     <row r="92">
       <c r="B92" s="48" t="inlineStr">
         <is>
-          <t>Заполняйте: каталог запчастей ТО (цена, кол-во, № ТО) и список узлов/капремонтов (стоимость по годам). КТГ, затраты ТО и капремонты пересчитаются снизу вверх; сводка «Данные по годам» и весь расчёт обновятся автоматически. Строка «Корректировка» и «Прочие/укрупнённо» — балансирующие, замените детализацией.</t>
+          <t>Заполняйте: каталог запчастей ТО (цена, кол-во, № ТО) и список узлов/капремонтов (нормо-час + стоимость по годам). Трудозатраты (сервис) считаются автоматически: нормо-часы ремонтируемых в году узлов × ставку (стр. «Ставка сервиса»); сервис ТО = ч·часы ТО × ставку. КТГ, затраты ТО и капремонты — снизу вверх; сводка «Данные по годам» и весь расчёт обновятся сами. Строки «Корректировка» и «Прочие/укрупнённо» — балансирующие.</t>
         </is>
       </c>
     </row>
@@ -18644,7 +18657,7 @@
     <row r="34">
       <c r="B34" s="37" t="inlineStr">
         <is>
-          <t>Капитальные ремонты (ППР) — из списка</t>
+          <t>Капитальные ремонты (запчасти) — авто</t>
         </is>
       </c>
       <c r="C34" s="24" t="inlineStr">
@@ -18653,50 +18666,50 @@
         </is>
       </c>
       <c r="E34" s="38">
-        <f>SUM(E69:E90)</f>
+        <f>SUM(E69:E90)-E35</f>
         <v/>
       </c>
       <c r="F34" s="38">
-        <f>SUM(F69:F90)</f>
+        <f>SUM(F69:F90)-F35</f>
         <v/>
       </c>
       <c r="G34" s="38">
-        <f>SUM(G69:G90)</f>
+        <f>SUM(G69:G90)-G35</f>
         <v/>
       </c>
       <c r="H34" s="38">
-        <f>SUM(H69:H90)</f>
+        <f>SUM(H69:H90)-H35</f>
         <v/>
       </c>
       <c r="I34" s="38">
-        <f>SUM(I69:I90)</f>
+        <f>SUM(I69:I90)-I35</f>
         <v/>
       </c>
       <c r="J34" s="38">
-        <f>SUM(J69:J90)</f>
+        <f>SUM(J69:J90)-J35</f>
         <v/>
       </c>
       <c r="K34" s="38">
-        <f>SUM(K69:K90)</f>
+        <f>SUM(K69:K90)-K35</f>
         <v/>
       </c>
       <c r="L34" s="38">
-        <f>SUM(L69:L90)</f>
+        <f>SUM(L69:L90)-L35</f>
         <v/>
       </c>
       <c r="M34" s="38">
-        <f>SUM(M69:M90)</f>
+        <f>SUM(M69:M90)-M35</f>
         <v/>
       </c>
       <c r="N34" s="38">
-        <f>SUM(N69:N90)</f>
+        <f>SUM(N69:N90)-N35</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="22" t="inlineStr">
-        <is>
-          <t>Сервис ремонтов (трудозатраты)</t>
+      <c r="B35" s="37" t="inlineStr">
+        <is>
+          <t>Сервис ремонтов (трудозатраты, авто)</t>
         </is>
       </c>
       <c r="C35" s="24" t="inlineStr">
@@ -18704,35 +18717,45 @@
           <t>тыс/год</t>
         </is>
       </c>
-      <c r="E35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" s="31" t="n">
-        <v>0</v>
+      <c r="E35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(E69:E90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="F35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(F69:F90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="G35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(G69:G90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="H35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(H69:H90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="I35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(I69:I90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="J35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(J69:J90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="K35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(K69:K90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="L35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(L69:L90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="M35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(M69:M90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="N35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(N69:N90&gt;0)*1)*$E$29/1000</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -19838,6 +19861,9 @@
           <t>Прочие/укрупнённо (капремонт)</t>
         </is>
       </c>
+      <c r="C90" s="47" t="n">
+        <v>250</v>
+      </c>
       <c r="E90" s="47" t="n">
         <v>0</v>
       </c>
@@ -19872,7 +19898,7 @@
     <row r="92">
       <c r="B92" s="48" t="inlineStr">
         <is>
-          <t>Заполняйте: каталог запчастей ТО (цена, кол-во, № ТО) и список узлов/капремонтов (стоимость по годам). КТГ, затраты ТО и капремонты пересчитаются снизу вверх; сводка «Данные по годам» и весь расчёт обновятся автоматически. Строка «Корректировка» и «Прочие/укрупнённо» — балансирующие, замените детализацией.</t>
+          <t>Заполняйте: каталог запчастей ТО (цена, кол-во, № ТО) и список узлов/капремонтов (нормо-час + стоимость по годам). Трудозатраты (сервис) считаются автоматически: нормо-часы ремонтируемых в году узлов × ставку (стр. «Ставка сервиса»); сервис ТО = ч·часы ТО × ставку. КТГ, затраты ТО и капремонты — снизу вверх; сводка «Данные по годам» и весь расчёт обновятся сами. Строки «Корректировка» и «Прочие/укрупнённо» — балансирующие.</t>
         </is>
       </c>
     </row>
@@ -20986,7 +21012,7 @@
     <row r="34">
       <c r="B34" s="37" t="inlineStr">
         <is>
-          <t>Капитальные ремонты (ППР) — из списка</t>
+          <t>Капитальные ремонты (запчасти) — авто</t>
         </is>
       </c>
       <c r="C34" s="24" t="inlineStr">
@@ -20995,50 +21021,50 @@
         </is>
       </c>
       <c r="E34" s="38">
-        <f>SUM(E69:E90)</f>
+        <f>SUM(E69:E90)-E35</f>
         <v/>
       </c>
       <c r="F34" s="38">
-        <f>SUM(F69:F90)</f>
+        <f>SUM(F69:F90)-F35</f>
         <v/>
       </c>
       <c r="G34" s="38">
-        <f>SUM(G69:G90)</f>
+        <f>SUM(G69:G90)-G35</f>
         <v/>
       </c>
       <c r="H34" s="38">
-        <f>SUM(H69:H90)</f>
+        <f>SUM(H69:H90)-H35</f>
         <v/>
       </c>
       <c r="I34" s="38">
-        <f>SUM(I69:I90)</f>
+        <f>SUM(I69:I90)-I35</f>
         <v/>
       </c>
       <c r="J34" s="38">
-        <f>SUM(J69:J90)</f>
+        <f>SUM(J69:J90)-J35</f>
         <v/>
       </c>
       <c r="K34" s="38">
-        <f>SUM(K69:K90)</f>
+        <f>SUM(K69:K90)-K35</f>
         <v/>
       </c>
       <c r="L34" s="38">
-        <f>SUM(L69:L90)</f>
+        <f>SUM(L69:L90)-L35</f>
         <v/>
       </c>
       <c r="M34" s="38">
-        <f>SUM(M69:M90)</f>
+        <f>SUM(M69:M90)-M35</f>
         <v/>
       </c>
       <c r="N34" s="38">
-        <f>SUM(N69:N90)</f>
+        <f>SUM(N69:N90)-N35</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="22" t="inlineStr">
-        <is>
-          <t>Сервис ремонтов (трудозатраты)</t>
+      <c r="B35" s="37" t="inlineStr">
+        <is>
+          <t>Сервис ремонтов (трудозатраты, авто)</t>
         </is>
       </c>
       <c r="C35" s="24" t="inlineStr">
@@ -21046,35 +21072,45 @@
           <t>тыс/год</t>
         </is>
       </c>
-      <c r="E35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" s="31" t="n">
-        <v>0</v>
+      <c r="E35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(E69:E90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="F35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(F69:F90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="G35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(G69:G90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="H35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(H69:H90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="I35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(I69:I90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="J35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(J69:J90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="K35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(K69:K90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="L35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(L69:L90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="M35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(M69:M90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="N35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(N69:N90&gt;0)*1)*$E$29/1000</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -22180,6 +22216,9 @@
           <t>Прочие/укрупнённо (капремонт)</t>
         </is>
       </c>
+      <c r="C90" s="47" t="n">
+        <v>250</v>
+      </c>
       <c r="E90" s="47" t="n">
         <v>0</v>
       </c>
@@ -22214,7 +22253,7 @@
     <row r="92">
       <c r="B92" s="48" t="inlineStr">
         <is>
-          <t>Заполняйте: каталог запчастей ТО (цена, кол-во, № ТО) и список узлов/капремонтов (стоимость по годам). КТГ, затраты ТО и капремонты пересчитаются снизу вверх; сводка «Данные по годам» и весь расчёт обновятся автоматически. Строка «Корректировка» и «Прочие/укрупнённо» — балансирующие, замените детализацией.</t>
+          <t>Заполняйте: каталог запчастей ТО (цена, кол-во, № ТО) и список узлов/капремонтов (нормо-час + стоимость по годам). Трудозатраты (сервис) считаются автоматически: нормо-часы ремонтируемых в году узлов × ставку (стр. «Ставка сервиса»); сервис ТО = ч·часы ТО × ставку. КТГ, затраты ТО и капремонты — снизу вверх; сводка «Данные по годам» и весь расчёт обновятся сами. Строки «Корректировка» и «Прочие/укрупнённо» — балансирующие.</t>
         </is>
       </c>
     </row>
@@ -23328,7 +23367,7 @@
     <row r="34">
       <c r="B34" s="37" t="inlineStr">
         <is>
-          <t>Капитальные ремонты (ППР) — из списка</t>
+          <t>Капитальные ремонты (запчасти) — авто</t>
         </is>
       </c>
       <c r="C34" s="24" t="inlineStr">
@@ -23337,50 +23376,50 @@
         </is>
       </c>
       <c r="E34" s="38">
-        <f>SUM(E69:E90)</f>
+        <f>SUM(E69:E90)-E35</f>
         <v/>
       </c>
       <c r="F34" s="38">
-        <f>SUM(F69:F90)</f>
+        <f>SUM(F69:F90)-F35</f>
         <v/>
       </c>
       <c r="G34" s="38">
-        <f>SUM(G69:G90)</f>
+        <f>SUM(G69:G90)-G35</f>
         <v/>
       </c>
       <c r="H34" s="38">
-        <f>SUM(H69:H90)</f>
+        <f>SUM(H69:H90)-H35</f>
         <v/>
       </c>
       <c r="I34" s="38">
-        <f>SUM(I69:I90)</f>
+        <f>SUM(I69:I90)-I35</f>
         <v/>
       </c>
       <c r="J34" s="38">
-        <f>SUM(J69:J90)</f>
+        <f>SUM(J69:J90)-J35</f>
         <v/>
       </c>
       <c r="K34" s="38">
-        <f>SUM(K69:K90)</f>
+        <f>SUM(K69:K90)-K35</f>
         <v/>
       </c>
       <c r="L34" s="38">
-        <f>SUM(L69:L90)</f>
+        <f>SUM(L69:L90)-L35</f>
         <v/>
       </c>
       <c r="M34" s="38">
-        <f>SUM(M69:M90)</f>
+        <f>SUM(M69:M90)-M35</f>
         <v/>
       </c>
       <c r="N34" s="38">
-        <f>SUM(N69:N90)</f>
+        <f>SUM(N69:N90)-N35</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="22" t="inlineStr">
-        <is>
-          <t>Сервис ремонтов (трудозатраты)</t>
+      <c r="B35" s="37" t="inlineStr">
+        <is>
+          <t>Сервис ремонтов (трудозатраты, авто)</t>
         </is>
       </c>
       <c r="C35" s="24" t="inlineStr">
@@ -23388,35 +23427,45 @@
           <t>тыс/год</t>
         </is>
       </c>
-      <c r="E35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" s="31" t="n">
-        <v>0</v>
+      <c r="E35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(E69:E90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="F35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(F69:F90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="G35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(G69:G90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="H35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(H69:H90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="I35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(I69:I90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="J35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(J69:J90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="K35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(K69:K90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="L35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(L69:L90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="M35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(M69:M90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="N35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(N69:N90&gt;0)*1)*$E$29/1000</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -24522,6 +24571,9 @@
           <t>Прочие/укрупнённо (капремонт)</t>
         </is>
       </c>
+      <c r="C90" s="47" t="n">
+        <v>250</v>
+      </c>
       <c r="E90" s="47" t="n">
         <v>0</v>
       </c>
@@ -24556,7 +24608,7 @@
     <row r="92">
       <c r="B92" s="48" t="inlineStr">
         <is>
-          <t>Заполняйте: каталог запчастей ТО (цена, кол-во, № ТО) и список узлов/капремонтов (стоимость по годам). КТГ, затраты ТО и капремонты пересчитаются снизу вверх; сводка «Данные по годам» и весь расчёт обновятся автоматически. Строка «Корректировка» и «Прочие/укрупнённо» — балансирующие, замените детализацией.</t>
+          <t>Заполняйте: каталог запчастей ТО (цена, кол-во, № ТО) и список узлов/капремонтов (нормо-час + стоимость по годам). Трудозатраты (сервис) считаются автоматически: нормо-часы ремонтируемых в году узлов × ставку (стр. «Ставка сервиса»); сервис ТО = ч·часы ТО × ставку. КТГ, затраты ТО и капремонты — снизу вверх; сводка «Данные по годам» и весь расчёт обновятся сами. Строки «Корректировка» и «Прочие/укрупнённо» — балансирующие.</t>
         </is>
       </c>
     </row>
@@ -25670,7 +25722,7 @@
     <row r="34">
       <c r="B34" s="37" t="inlineStr">
         <is>
-          <t>Капитальные ремонты (ППР) — из списка</t>
+          <t>Капитальные ремонты (запчасти) — авто</t>
         </is>
       </c>
       <c r="C34" s="24" t="inlineStr">
@@ -25679,50 +25731,50 @@
         </is>
       </c>
       <c r="E34" s="38">
-        <f>SUM(E69:E90)</f>
+        <f>SUM(E69:E90)-E35</f>
         <v/>
       </c>
       <c r="F34" s="38">
-        <f>SUM(F69:F90)</f>
+        <f>SUM(F69:F90)-F35</f>
         <v/>
       </c>
       <c r="G34" s="38">
-        <f>SUM(G69:G90)</f>
+        <f>SUM(G69:G90)-G35</f>
         <v/>
       </c>
       <c r="H34" s="38">
-        <f>SUM(H69:H90)</f>
+        <f>SUM(H69:H90)-H35</f>
         <v/>
       </c>
       <c r="I34" s="38">
-        <f>SUM(I69:I90)</f>
+        <f>SUM(I69:I90)-I35</f>
         <v/>
       </c>
       <c r="J34" s="38">
-        <f>SUM(J69:J90)</f>
+        <f>SUM(J69:J90)-J35</f>
         <v/>
       </c>
       <c r="K34" s="38">
-        <f>SUM(K69:K90)</f>
+        <f>SUM(K69:K90)-K35</f>
         <v/>
       </c>
       <c r="L34" s="38">
-        <f>SUM(L69:L90)</f>
+        <f>SUM(L69:L90)-L35</f>
         <v/>
       </c>
       <c r="M34" s="38">
-        <f>SUM(M69:M90)</f>
+        <f>SUM(M69:M90)-M35</f>
         <v/>
       </c>
       <c r="N34" s="38">
-        <f>SUM(N69:N90)</f>
+        <f>SUM(N69:N90)-N35</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="22" t="inlineStr">
-        <is>
-          <t>Сервис ремонтов (трудозатраты)</t>
+      <c r="B35" s="37" t="inlineStr">
+        <is>
+          <t>Сервис ремонтов (трудозатраты, авто)</t>
         </is>
       </c>
       <c r="C35" s="24" t="inlineStr">
@@ -25730,35 +25782,45 @@
           <t>тыс/год</t>
         </is>
       </c>
-      <c r="E35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" s="31" t="n">
-        <v>0</v>
+      <c r="E35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(E69:E90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="F35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(F69:F90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="G35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(G69:G90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="H35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(H69:H90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="I35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(I69:I90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="J35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(J69:J90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="K35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(K69:K90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="L35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(L69:L90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="M35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(M69:M90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="N35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(N69:N90&gt;0)*1)*$E$29/1000</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -26864,6 +26926,9 @@
           <t>Прочие/укрупнённо (капремонт)</t>
         </is>
       </c>
+      <c r="C90" s="47" t="n">
+        <v>250</v>
+      </c>
       <c r="E90" s="47" t="n">
         <v>0</v>
       </c>
@@ -26898,7 +26963,7 @@
     <row r="92">
       <c r="B92" s="48" t="inlineStr">
         <is>
-          <t>Заполняйте: каталог запчастей ТО (цена, кол-во, № ТО) и список узлов/капремонтов (стоимость по годам). КТГ, затраты ТО и капремонты пересчитаются снизу вверх; сводка «Данные по годам» и весь расчёт обновятся автоматически. Строка «Корректировка» и «Прочие/укрупнённо» — балансирующие, замените детализацией.</t>
+          <t>Заполняйте: каталог запчастей ТО (цена, кол-во, № ТО) и список узлов/капремонтов (нормо-час + стоимость по годам). Трудозатраты (сервис) считаются автоматически: нормо-часы ремонтируемых в году узлов × ставку (стр. «Ставка сервиса»); сервис ТО = ч·часы ТО × ставку. КТГ, затраты ТО и капремонты — снизу вверх; сводка «Данные по годам» и весь расчёт обновятся сами. Строки «Корректировка» и «Прочие/укрупнённо» — балансирующие.</t>
         </is>
       </c>
     </row>
@@ -28012,7 +28077,7 @@
     <row r="34">
       <c r="B34" s="37" t="inlineStr">
         <is>
-          <t>Капитальные ремонты (ППР) — из списка</t>
+          <t>Капитальные ремонты (запчасти) — авто</t>
         </is>
       </c>
       <c r="C34" s="24" t="inlineStr">
@@ -28021,50 +28086,50 @@
         </is>
       </c>
       <c r="E34" s="38">
-        <f>SUM(E69:E90)</f>
+        <f>SUM(E69:E90)-E35</f>
         <v/>
       </c>
       <c r="F34" s="38">
-        <f>SUM(F69:F90)</f>
+        <f>SUM(F69:F90)-F35</f>
         <v/>
       </c>
       <c r="G34" s="38">
-        <f>SUM(G69:G90)</f>
+        <f>SUM(G69:G90)-G35</f>
         <v/>
       </c>
       <c r="H34" s="38">
-        <f>SUM(H69:H90)</f>
+        <f>SUM(H69:H90)-H35</f>
         <v/>
       </c>
       <c r="I34" s="38">
-        <f>SUM(I69:I90)</f>
+        <f>SUM(I69:I90)-I35</f>
         <v/>
       </c>
       <c r="J34" s="38">
-        <f>SUM(J69:J90)</f>
+        <f>SUM(J69:J90)-J35</f>
         <v/>
       </c>
       <c r="K34" s="38">
-        <f>SUM(K69:K90)</f>
+        <f>SUM(K69:K90)-K35</f>
         <v/>
       </c>
       <c r="L34" s="38">
-        <f>SUM(L69:L90)</f>
+        <f>SUM(L69:L90)-L35</f>
         <v/>
       </c>
       <c r="M34" s="38">
-        <f>SUM(M69:M90)</f>
+        <f>SUM(M69:M90)-M35</f>
         <v/>
       </c>
       <c r="N34" s="38">
-        <f>SUM(N69:N90)</f>
+        <f>SUM(N69:N90)-N35</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="22" t="inlineStr">
-        <is>
-          <t>Сервис ремонтов (трудозатраты)</t>
+      <c r="B35" s="37" t="inlineStr">
+        <is>
+          <t>Сервис ремонтов (трудозатраты, авто)</t>
         </is>
       </c>
       <c r="C35" s="24" t="inlineStr">
@@ -28072,35 +28137,45 @@
           <t>тыс/год</t>
         </is>
       </c>
-      <c r="E35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" s="31" t="n">
-        <v>0</v>
+      <c r="E35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(E69:E90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="F35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(F69:F90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="G35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(G69:G90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="H35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(H69:H90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="I35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(I69:I90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="J35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(J69:J90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="K35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(K69:K90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="L35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(L69:L90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="M35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(M69:M90&gt;0)*1)*$E$29/1000</f>
+        <v/>
+      </c>
+      <c r="N35" s="38">
+        <f>SUMPRODUCT($C$69:$C$90,(N69:N90&gt;0)*1)*$E$29/1000</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -29206,6 +29281,9 @@
           <t>Прочие/укрупнённо (капремонт)</t>
         </is>
       </c>
+      <c r="C90" s="47" t="n">
+        <v>250</v>
+      </c>
       <c r="E90" s="47" t="n">
         <v>0</v>
       </c>
@@ -29240,7 +29318,7 @@
     <row r="92">
       <c r="B92" s="48" t="inlineStr">
         <is>
-          <t>Заполняйте: каталог запчастей ТО (цена, кол-во, № ТО) и список узлов/капремонтов (стоимость по годам). КТГ, затраты ТО и капремонты пересчитаются снизу вверх; сводка «Данные по годам» и весь расчёт обновятся автоматически. Строка «Корректировка» и «Прочие/укрупнённо» — балансирующие, замените детализацией.</t>
+          <t>Заполняйте: каталог запчастей ТО (цена, кол-во, № ТО) и список узлов/капремонтов (нормо-час + стоимость по годам). Трудозатраты (сервис) считаются автоматически: нормо-часы ремонтируемых в году узлов × ставку (стр. «Ставка сервиса»); сервис ТО = ч·часы ТО × ставку. КТГ, затраты ТО и капремонты — снизу вверх; сводка «Данные по годам» и весь расчёт обновятся сами. Строки «Корректировка» и «Прочие/укрупнённо» — балансирующие.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add explicit per-shift maintenance (20 min/shift) and verify productivity
- Per-shift daily maintenance (ежесменное ТО, 20 min per 12h shift) is now an
  explicit, auto-computed downtime line in each template, matching the supplier
  'Данные_Экскаватор' formula: (КФВ - ТО downtime - repair downtime)/shift x 20/60.
  Repair downtime is recalibrated so КТГ still matches the reference model.
- Verified productivity against the big model: PC2000-8 year-1 output = 2213.5
  тыс.м3 (m3/h 433.76, effective time 5103 h), identical to sheet '2. Произв-сть'.
- Full workbook recalculates with zero errors; annuities unchanged (PC2000-8
  48.71 руб/м3); downtime split reconciles (273 ТО + 161 repair + 231 daily = 665 h).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WL5xBBk55GzPMRGQKQMRy3
</commit_message>
<xml_diff>
--- a/Модель_TCO_экскаваторов_аннуитет.xlsx
+++ b/Модель_TCO_экскаваторов_аннуитет.xlsx
@@ -2606,9 +2606,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="22" t="inlineStr">
-        <is>
-          <t>Ежесменный осмотр</t>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>Ежесменное ТО (20 мин/смену)</t>
         </is>
       </c>
       <c r="C10" s="24" t="inlineStr">
@@ -2616,35 +2616,45 @@
           <t>ч/год</t>
         </is>
       </c>
-      <c r="E10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="31" t="n">
-        <v>0</v>
+      <c r="E10" s="38">
+        <f>('Параметры'!C26-E8-E9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="F10" s="38">
+        <f>('Параметры'!C26-F8-F9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="G10" s="38">
+        <f>('Параметры'!C26-G8-G9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="H10" s="38">
+        <f>('Параметры'!C26-H8-H9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="I10" s="38">
+        <f>('Параметры'!C26-I8-I9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="J10" s="38">
+        <f>('Параметры'!C26-J8-J9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="K10" s="38">
+        <f>('Параметры'!C26-K8-K9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="L10" s="38">
+        <f>('Параметры'!C26-L8-L9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="M10" s="38">
+        <f>('Параметры'!C26-M8-M9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="N10" s="38">
+        <f>('Параметры'!C26-N8-N9)/'Параметры'!C33*20/60</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -3347,34 +3357,34 @@
         </is>
       </c>
       <c r="E32" s="31" t="n">
-        <v>1000.04</v>
+        <v>786.13</v>
       </c>
       <c r="F32" s="31" t="n">
-        <v>2106.65</v>
+        <v>1924.36</v>
       </c>
       <c r="G32" s="31" t="n">
-        <v>1871.91</v>
+        <v>1682.92</v>
       </c>
       <c r="H32" s="31" t="n">
-        <v>2402.67</v>
+        <v>2228.84</v>
       </c>
       <c r="I32" s="31" t="n">
-        <v>2412.57</v>
+        <v>2239.02</v>
       </c>
       <c r="J32" s="31" t="n">
-        <v>1980.41</v>
+        <v>1794.52</v>
       </c>
       <c r="K32" s="31" t="n">
-        <v>2204.54</v>
+        <v>2025.05</v>
       </c>
       <c r="L32" s="31" t="n">
-        <v>1713.31</v>
+        <v>1519.78</v>
       </c>
       <c r="M32" s="31" t="n">
-        <v>2635.37</v>
+        <v>2468.19</v>
       </c>
       <c r="N32" s="31" t="n">
-        <v>1852.89</v>
+        <v>1663.35</v>
       </c>
     </row>
     <row r="33">
@@ -17841,9 +17851,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="22" t="inlineStr">
-        <is>
-          <t>Ежесменный осмотр</t>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>Ежесменное ТО (20 мин/смену)</t>
         </is>
       </c>
       <c r="C10" s="24" t="inlineStr">
@@ -17851,35 +17861,45 @@
           <t>ч/год</t>
         </is>
       </c>
-      <c r="E10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="31" t="n">
-        <v>0</v>
+      <c r="E10" s="38">
+        <f>('Параметры'!C26-E8-E9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="F10" s="38">
+        <f>('Параметры'!C26-F8-F9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="G10" s="38">
+        <f>('Параметры'!C26-G8-G9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="H10" s="38">
+        <f>('Параметры'!C26-H8-H9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="I10" s="38">
+        <f>('Параметры'!C26-I8-I9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="J10" s="38">
+        <f>('Параметры'!C26-J8-J9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="K10" s="38">
+        <f>('Параметры'!C26-K8-K9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="L10" s="38">
+        <f>('Параметры'!C26-L8-L9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="M10" s="38">
+        <f>('Параметры'!C26-M8-M9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="N10" s="38">
+        <f>('Параметры'!C26-N8-N9)/'Параметры'!C33*20/60</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -18582,34 +18602,34 @@
         </is>
       </c>
       <c r="E32" s="31" t="n">
-        <v>392</v>
+        <v>160.72</v>
       </c>
       <c r="F32" s="31" t="n">
-        <v>602.79</v>
+        <v>377.53</v>
       </c>
       <c r="G32" s="31" t="n">
-        <v>953.1900000000001</v>
+        <v>737.9400000000001</v>
       </c>
       <c r="H32" s="31" t="n">
-        <v>1040.79</v>
+        <v>828.05</v>
       </c>
       <c r="I32" s="31" t="n">
-        <v>953.1900000000001</v>
+        <v>737.9400000000001</v>
       </c>
       <c r="J32" s="31" t="n">
-        <v>1372.37</v>
+        <v>1169.1</v>
       </c>
       <c r="K32" s="31" t="n">
-        <v>1596.5</v>
+        <v>1399.63</v>
       </c>
       <c r="L32" s="31" t="n">
-        <v>1105.27</v>
+        <v>894.37</v>
       </c>
       <c r="M32" s="31" t="n">
-        <v>2027.33</v>
+        <v>1842.78</v>
       </c>
       <c r="N32" s="31" t="n">
-        <v>1244.85</v>
+        <v>1037.94</v>
       </c>
     </row>
     <row r="33">
@@ -20196,9 +20216,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="22" t="inlineStr">
-        <is>
-          <t>Ежесменный осмотр</t>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>Ежесменное ТО (20 мин/смену)</t>
         </is>
       </c>
       <c r="C10" s="24" t="inlineStr">
@@ -20206,35 +20226,45 @@
           <t>ч/год</t>
         </is>
       </c>
-      <c r="E10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="31" t="n">
-        <v>0</v>
+      <c r="E10" s="38">
+        <f>('Параметры'!C26-E8-E9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="F10" s="38">
+        <f>('Параметры'!C26-F8-F9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="G10" s="38">
+        <f>('Параметры'!C26-G8-G9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="H10" s="38">
+        <f>('Параметры'!C26-H8-H9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="I10" s="38">
+        <f>('Параметры'!C26-I8-I9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="J10" s="38">
+        <f>('Параметры'!C26-J8-J9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="K10" s="38">
+        <f>('Параметры'!C26-K8-K9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="L10" s="38">
+        <f>('Параметры'!C26-L8-L9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="M10" s="38">
+        <f>('Параметры'!C26-M8-M9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="N10" s="38">
+        <f>('Параметры'!C26-N8-N9)/'Параметры'!C33*20/60</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -20937,34 +20967,34 @@
         </is>
       </c>
       <c r="E32" s="31" t="n">
-        <v>392</v>
+        <v>160.72</v>
       </c>
       <c r="F32" s="31" t="n">
-        <v>1498.61</v>
+        <v>1298.94</v>
       </c>
       <c r="G32" s="31" t="n">
-        <v>1263.87</v>
+        <v>1057.5</v>
       </c>
       <c r="H32" s="31" t="n">
-        <v>1794.64</v>
+        <v>1603.44</v>
       </c>
       <c r="I32" s="31" t="n">
-        <v>1804.53</v>
+        <v>1613.61</v>
       </c>
       <c r="J32" s="31" t="n">
-        <v>1372.37</v>
+        <v>1169.1</v>
       </c>
       <c r="K32" s="31" t="n">
-        <v>1596.5</v>
+        <v>1399.63</v>
       </c>
       <c r="L32" s="31" t="n">
-        <v>1105.27</v>
+        <v>894.37</v>
       </c>
       <c r="M32" s="31" t="n">
-        <v>2027.33</v>
+        <v>1842.78</v>
       </c>
       <c r="N32" s="31" t="n">
-        <v>1244.85</v>
+        <v>1037.94</v>
       </c>
     </row>
     <row r="33">
@@ -22551,9 +22581,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="22" t="inlineStr">
-        <is>
-          <t>Ежесменный осмотр</t>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>Ежесменное ТО (20 мин/смену)</t>
         </is>
       </c>
       <c r="C10" s="24" t="inlineStr">
@@ -22561,35 +22591,45 @@
           <t>ч/год</t>
         </is>
       </c>
-      <c r="E10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="31" t="n">
-        <v>0</v>
+      <c r="E10" s="38">
+        <f>('Параметры'!C26-E8-E9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="F10" s="38">
+        <f>('Параметры'!C26-F8-F9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="G10" s="38">
+        <f>('Параметры'!C26-G8-G9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="H10" s="38">
+        <f>('Параметры'!C26-H8-H9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="I10" s="38">
+        <f>('Параметры'!C26-I8-I9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="J10" s="38">
+        <f>('Параметры'!C26-J8-J9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="K10" s="38">
+        <f>('Параметры'!C26-K8-K9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="L10" s="38">
+        <f>('Параметры'!C26-L8-L9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="M10" s="38">
+        <f>('Параметры'!C26-M8-M9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="N10" s="38">
+        <f>('Параметры'!C26-N8-N9)/'Параметры'!C33*20/60</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -23292,34 +23332,34 @@
         </is>
       </c>
       <c r="E32" s="31" t="n">
-        <v>1000.04</v>
+        <v>786.13</v>
       </c>
       <c r="F32" s="31" t="n">
-        <v>2106.65</v>
+        <v>1924.36</v>
       </c>
       <c r="G32" s="31" t="n">
-        <v>1871.91</v>
+        <v>1682.92</v>
       </c>
       <c r="H32" s="31" t="n">
-        <v>2402.67</v>
+        <v>2228.84</v>
       </c>
       <c r="I32" s="31" t="n">
-        <v>2412.57</v>
+        <v>2239.02</v>
       </c>
       <c r="J32" s="31" t="n">
-        <v>1980.41</v>
+        <v>1794.52</v>
       </c>
       <c r="K32" s="31" t="n">
-        <v>2204.54</v>
+        <v>2025.05</v>
       </c>
       <c r="L32" s="31" t="n">
-        <v>1713.31</v>
+        <v>1519.78</v>
       </c>
       <c r="M32" s="31" t="n">
-        <v>2635.37</v>
+        <v>2468.19</v>
       </c>
       <c r="N32" s="31" t="n">
-        <v>1852.89</v>
+        <v>1663.35</v>
       </c>
     </row>
     <row r="33">
@@ -24906,9 +24946,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="22" t="inlineStr">
-        <is>
-          <t>Ежесменный осмотр</t>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>Ежесменное ТО (20 мин/смену)</t>
         </is>
       </c>
       <c r="C10" s="24" t="inlineStr">
@@ -24916,35 +24956,45 @@
           <t>ч/год</t>
         </is>
       </c>
-      <c r="E10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="31" t="n">
-        <v>0</v>
+      <c r="E10" s="38">
+        <f>('Параметры'!C26-E8-E9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="F10" s="38">
+        <f>('Параметры'!C26-F8-F9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="G10" s="38">
+        <f>('Параметры'!C26-G8-G9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="H10" s="38">
+        <f>('Параметры'!C26-H8-H9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="I10" s="38">
+        <f>('Параметры'!C26-I8-I9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="J10" s="38">
+        <f>('Параметры'!C26-J8-J9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="K10" s="38">
+        <f>('Параметры'!C26-K8-K9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="L10" s="38">
+        <f>('Параметры'!C26-L8-L9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="M10" s="38">
+        <f>('Параметры'!C26-M8-M9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="N10" s="38">
+        <f>('Параметры'!C26-N8-N9)/'Параметры'!C33*20/60</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -25647,34 +25697,34 @@
         </is>
       </c>
       <c r="E32" s="31" t="n">
-        <v>1000.04</v>
+        <v>786.13</v>
       </c>
       <c r="F32" s="31" t="n">
-        <v>2106.65</v>
+        <v>1924.36</v>
       </c>
       <c r="G32" s="31" t="n">
-        <v>1871.91</v>
+        <v>1682.92</v>
       </c>
       <c r="H32" s="31" t="n">
-        <v>2402.67</v>
+        <v>2228.84</v>
       </c>
       <c r="I32" s="31" t="n">
-        <v>2412.57</v>
+        <v>2239.02</v>
       </c>
       <c r="J32" s="31" t="n">
-        <v>1980.41</v>
+        <v>1794.52</v>
       </c>
       <c r="K32" s="31" t="n">
-        <v>2204.54</v>
+        <v>2025.05</v>
       </c>
       <c r="L32" s="31" t="n">
-        <v>1713.31</v>
+        <v>1519.78</v>
       </c>
       <c r="M32" s="31" t="n">
-        <v>2635.37</v>
+        <v>2468.19</v>
       </c>
       <c r="N32" s="31" t="n">
-        <v>1852.89</v>
+        <v>1663.35</v>
       </c>
     </row>
     <row r="33">
@@ -27261,9 +27311,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="22" t="inlineStr">
-        <is>
-          <t>Ежесменный осмотр</t>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>Ежесменное ТО (20 мин/смену)</t>
         </is>
       </c>
       <c r="C10" s="24" t="inlineStr">
@@ -27271,35 +27321,45 @@
           <t>ч/год</t>
         </is>
       </c>
-      <c r="E10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="31" t="n">
-        <v>0</v>
+      <c r="E10" s="38">
+        <f>('Параметры'!C26-E8-E9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="F10" s="38">
+        <f>('Параметры'!C26-F8-F9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="G10" s="38">
+        <f>('Параметры'!C26-G8-G9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="H10" s="38">
+        <f>('Параметры'!C26-H8-H9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="I10" s="38">
+        <f>('Параметры'!C26-I8-I9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="J10" s="38">
+        <f>('Параметры'!C26-J8-J9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="K10" s="38">
+        <f>('Параметры'!C26-K8-K9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="L10" s="38">
+        <f>('Параметры'!C26-L8-L9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="M10" s="38">
+        <f>('Параметры'!C26-M8-M9)/'Параметры'!C33*20/60</f>
+        <v/>
+      </c>
+      <c r="N10" s="38">
+        <f>('Параметры'!C26-N8-N9)/'Параметры'!C33*20/60</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -28002,34 +28062,34 @@
         </is>
       </c>
       <c r="E32" s="31" t="n">
-        <v>1000.04</v>
+        <v>786.13</v>
       </c>
       <c r="F32" s="31" t="n">
-        <v>2106.65</v>
+        <v>1924.36</v>
       </c>
       <c r="G32" s="31" t="n">
-        <v>1871.91</v>
+        <v>1682.92</v>
       </c>
       <c r="H32" s="31" t="n">
-        <v>2402.67</v>
+        <v>2228.84</v>
       </c>
       <c r="I32" s="31" t="n">
-        <v>2412.57</v>
+        <v>2239.02</v>
       </c>
       <c r="J32" s="31" t="n">
-        <v>1980.41</v>
+        <v>1794.52</v>
       </c>
       <c r="K32" s="31" t="n">
-        <v>2204.54</v>
+        <v>2025.05</v>
       </c>
       <c r="L32" s="31" t="n">
-        <v>1713.31</v>
+        <v>1519.78</v>
       </c>
       <c r="M32" s="31" t="n">
-        <v>2635.37</v>
+        <v>2468.19</v>
       </c>
       <c r="N32" s="31" t="n">
-        <v>1852.89</v>
+        <v>1663.35</v>
       </c>
     </row>
     <row r="33">

</xml_diff>